<commit_message>
Vérification des chiffres des classeurs ; TVA : perte de pouvoir d'achat lue sur le graphique 4 du Trésor-Éco
- TVA sociale : la perte par point de taux normal n'est plus le prorata 0,5 % × 8,9 / 13,7 (0,325 %) mais les
  valeurs du graphique 4 du Trésor-Éco n° 371, par cinquième de niveau de vie (0,39 % à 0,25 % ; moyenne 0,30 %),
  avec le choix du cinquième dans le simulateur et le classeur.
- Classeurs : feuille « Vérification » (type, calcul, source, lien, statut de chaque chiffre saisi), colonnes « Type »
  et « Comment c'est calculé » dans les tableaux de paramètres, source Insee dans la feuille Niveaux de vie.
- Registre tools/chiffrages/verification.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188qNw1StBQkFA1rFcQwdyx
</commit_message>
<xml_diff>
--- a/site/chiffrages/Chiffrage_Heritage.xlsx
+++ b/site/chiffrages/Chiffrage_Heritage.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Calcul individuel" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Gain salaire" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Sources" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Vérification" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="223">
   <si>
     <t xml:space="preserve">Chiffrage de l'espace Héritage</t>
   </si>
@@ -85,6 +86,9 @@
     <t xml:space="preserve">L'étude mêle euros courants et croissances réelles (PIB +1 %/an sans inflation) ; la part du top 1 % du patrimoine y passe de 24 % à 35 % en 2040 ; aucun effet de comportement (exil, optimisation, étalement du paiement).</t>
   </si>
   <si>
+    <t xml:space="preserve">Chaque chiffre saisi est revérifié à la source : voir la feuille « Vérification » (type, calcul, source, statut).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Légende des couleurs</t>
   </si>
   <si>
@@ -133,39 +137,75 @@
     <t xml:space="preserve">Source</t>
   </si>
   <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment c'est calculé</t>
+  </si>
+  <si>
     <t xml:space="preserve">Croissance annuelle du PIB (après la dernière année connue)</t>
   </si>
   <si>
     <t xml:space="preserve">Étude : +1 % par an</t>
   </si>
   <si>
+    <t xml:space="preserve">Hypothèse du site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypothèse de l'étude : +1 % par an après la dernière année connue.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Flux successoral en 2050 (part du PIB)</t>
   </si>
   <si>
     <t xml:space="preserve">CAE, note n° 63, 2021 (d'après Goupille-Lebret et al.)</t>
   </si>
   <si>
+    <t xml:space="preserve">Chiffre publié</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 % du PIB en 2050 (CAE, note n° 63) ; interpolation linéaire depuis 15 % en 2021.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Croissance annuelle du patrimoine du top 1 %</t>
   </si>
   <si>
     <t xml:space="preserve">Garbinti, Goupille-Lebret et Piketty (2021) : 6,10 % par an en moyenne sur 2005-2014, moins 2 % d'inflation</t>
   </si>
   <si>
+    <t xml:space="preserve">Calcul du site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,10 % de rendement moyen 2005-2014 (Garbinti et al.) − 2 % d'inflation.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part de plus-values latentes dans le patrimoine du top 1 %</t>
   </si>
   <si>
     <t xml:space="preserve">Saez et al. (2021) : 17 681 Md€ de plus-values latentes sur 42 861 Md€ de patrimoine du top 1 %</t>
   </si>
   <si>
+    <t xml:space="preserve">17 681 Md€ de plus-values latentes ÷ 42 861 Md€ de patrimoine du top 1 % (Saez et al.).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Taux du PFU</t>
   </si>
   <si>
     <t xml:space="preserve">PFU de 30 % (2024) / PFU de 31,4 % depuis le 1er janvier 2026 (12,8 % d'impôt + 18,6 % de prélèvements sociaux, LFSS 2026)</t>
   </si>
   <si>
+    <t xml:space="preserve">Loi ou barème</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 % en 2024 ; 31,4 % depuis 2026 (12,8 % + 18,6 %).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Flux successoral en 2021 (part du PIB)</t>
   </si>
   <si>
+    <t xml:space="preserve">15 % du PIB en 2021 (CAE, note n° 63).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Année de départ du flux</t>
   </si>
   <si>
@@ -178,12 +218,18 @@
     <t xml:space="preserve">CAE (2021), simulation de la réforme de l'assiette et du barème, reprise par l'étude</t>
   </si>
   <si>
+    <t xml:space="preserve">10 Md€ en 2021 (simulation du CAE reprise par l'étude), puis comme le flux successoral.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part du patrimoine détenue par le top 1 % (année de référence)</t>
   </si>
   <si>
     <t xml:space="preserve">World Inequality Database, 2022</t>
   </si>
   <si>
+    <t xml:space="preserve">24 % (World Inequality Database, 2022).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Année de référence du patrimoine du top 1 %</t>
   </si>
   <si>
@@ -193,18 +239,27 @@
     <t xml:space="preserve">4,07 % − 2 % d'inflation (étude, Banque de France)</t>
   </si>
   <si>
+    <t xml:space="preserve">4,07 % − 2 % d'inflation (classeur de l'étude, Banque de France).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part de l'assiette taxée après abattements</t>
   </si>
   <si>
     <t xml:space="preserve">Hannezo et al. (2022)</t>
   </si>
   <si>
+    <t xml:space="preserve">80 % de l'assiette taxée (Hannezo et al., 2022).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réduction pour droits de succession déjà payés</t>
   </si>
   <si>
     <t xml:space="preserve">CAE (2021)</t>
   </si>
   <si>
+    <t xml:space="preserve">20 % de droits déjà payés déduits (CAE, 2021).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Données connues par année (au-delà : projection)</t>
   </si>
   <si>
@@ -518,6 +573,150 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.insee.fr/fr/statistiques/8574681?sommaire=8574832</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérification des chiffres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chaque chiffre saisi dans ce classeur, revérifié à la source en octobre 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remarque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème en ligne directe (5 % à 45 %, tranches de 8 072 à 1 805 677 €) et abattement de 100 000 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème légal, inchangé depuis 2011.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGI, art. 777 et 779</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.legifrance.gouv.fr/codes/texte_lc/LEGITEXT000006069577</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'étude écrit « 15 392 € » pour la borne de la tranche à 15 % ; le bon chiffre, retenu ici, est 15 932 €.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assurance-vie : abattement de 152 500 € par bénéficiaire, 20 % jusqu'à 700 000 €, 31,25 % au-delà</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primes versées avant 70 ans.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGI, art. 990 I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème de l'IGS (0 % jusqu'à 200 000 €, puis 5 / 15 / 25 / 35 / 45 / 50 %)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau 6 de l'étude (proposition du CAE, 2021).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fondation Jean-Jaurès (2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PFU sur les plus-values latentes (calcul individuel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux de l'étude (2024) ; 31,4 % depuis 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flux successoral, pilier 1, pilier 2 : formules et hypothèses du scénario « Étude 2024 »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repris du classeur de chiffrage de l'étude, cellule par cellule (vérifié : mêmes résultats à 0,01 Md€ près).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fondation Jean-Jaurès (2024), classeur « Chiffrage IGS »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIB 2025 (scénario actualisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 991,1 Md€</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024 déduit : 2 991,1 ÷ 1,019 (croissance en valeur de 1,9 %).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insee, Les comptes de la Nation en 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Droits de succession et donations 2024-2026 (scénario actualisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20,9 ; 20,7 ; 21,4 Md€</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donations + successions : 4,9 + 16,0 ; 4,5 + 16,2 ; 4,4 + 17,0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voies et moyens, PLF 2026, tome I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrimoine net des ménages (scénario actualisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 953 Md€ fin 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023 et 2022 déduits des évolutions publiées (+0,7 %, +0,6 %).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insee Première n° 2081</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PFU (scénario actualisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31,4 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12,8 % d'impôt + 18,6 % de prélèvements sociaux depuis le 1er janvier 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LFSS 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://placement.meilleurtaux.com/placement-financier/actualites/2026-avril/flat-tax-a-31-4-ce-qui-change-depuis-janvier-2026.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnes en emploi ; salaires bruts ; ratio net / brut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30,4 M ; 1 108,5 Md€ ; 78 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voir le classeur Retraites (ratio : hypothèse du site).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.insee.fr/fr/statistiques/8376894</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Types : « Chiffre publié » (repris d'une publication), « Lu sur un graphique », « Calcul du site » (formule à partir de chiffres publiés), « Hypothèse du site », « Loi ou barème ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statuts : « Confirmé » (vérifié à la source primaire), « Corrigé » (valeur changée lors de cette vérification), « Confirmé (source secondaire) », « Estimation, non vérifiable ».</t>
   </si>
 </sst>
 </file>
@@ -695,7 +894,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -716,6 +915,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -724,10 +927,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -882,6 +1081,10 @@
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1136,7 +1339,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1203,33 +1406,38 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1248,62 +1456,70 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="B4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="n">
         <f aca="false">IF(B4="Étude 2024",1,2)</f>
         <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>0.01</v>
@@ -1317,12 +1533,18 @@
         <v>0.01</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>32</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>0.23</v>
@@ -1336,12 +1558,18 @@
         <v>0.23</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>0.041</v>
@@ -1355,12 +1583,18 @@
         <v>0.041</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>40</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>0.412519539908075</v>
@@ -1374,12 +1608,18 @@
         <v>0.412519539908075</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>35</v>
+        <v>44</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>0.3</v>
@@ -1393,12 +1633,18 @@
         <v>0.314</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>37</v>
+        <v>47</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="B12" s="11" t="n">
         <v>0.15</v>
@@ -1412,12 +1658,18 @@
         <v>0.15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>31</v>
+        <v>36</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>2021</v>
@@ -1431,10 +1683,14 @@
         <v>2021</v>
       </c>
       <c r="F13" s="4"/>
+      <c r="G13" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>2050</v>
@@ -1448,10 +1704,14 @@
         <v>2050</v>
       </c>
       <c r="F14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G14" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B15" s="20" t="n">
         <v>10</v>
@@ -1465,12 +1725,18 @@
         <v>10</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>42</v>
+        <v>55</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>0.24</v>
@@ -1484,12 +1750,18 @@
         <v>0.24</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>44</v>
+        <v>58</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>2022</v>
@@ -1503,10 +1775,14 @@
         <v>2022</v>
       </c>
       <c r="F17" s="4"/>
+      <c r="G17" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>0.0207</v>
@@ -1520,12 +1796,18 @@
         <v>0.0207</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>47</v>
+        <v>62</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="B19" s="11" t="n">
         <v>0.8</v>
@@ -1539,12 +1821,18 @@
         <v>0.8</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>49</v>
+        <v>65</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="B20" s="11" t="n">
         <v>0.2</v>
@@ -1558,35 +1846,41 @@
         <v>0.2</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>51</v>
+        <v>68</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>55</v>
+      <c r="A24" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>2021</v>
@@ -1598,12 +1892,12 @@
         <v>2508.1023</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>55</v>
+      <c r="A25" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B25" s="17" t="n">
         <v>2022</v>
@@ -1615,12 +1909,12 @@
         <v>2655.435</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>55</v>
+      <c r="A26" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B26" s="17" t="n">
         <v>2023</v>
@@ -1632,12 +1926,12 @@
         <v>2822.5</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
-        <v>55</v>
+      <c r="A27" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B27" s="17" t="n">
         <v>2024</v>
@@ -1646,12 +1940,12 @@
         <v>2935.32875368008</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>55</v>
+      <c r="A28" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B28" s="17" t="n">
         <v>2025</v>
@@ -1660,12 +1954,12 @@
         <v>2991.1</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
-        <v>57</v>
+      <c r="A29" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B29" s="17" t="n">
         <v>2021</v>
@@ -1677,12 +1971,12 @@
         <v>18.7</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
-        <v>57</v>
+      <c r="A30" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B30" s="17" t="n">
         <v>2022</v>
@@ -1694,12 +1988,12 @@
         <v>18.7</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
-        <v>57</v>
+      <c r="A31" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B31" s="17" t="n">
         <v>2023</v>
@@ -1711,12 +2005,12 @@
         <v>20.8</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>57</v>
+      <c r="A32" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B32" s="17" t="n">
         <v>2024</v>
@@ -1725,12 +2019,12 @@
         <v>20.9</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>57</v>
+      <c r="A33" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B33" s="17" t="n">
         <v>2025</v>
@@ -1739,12 +2033,12 @@
         <v>20.7</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
-        <v>57</v>
+      <c r="A34" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B34" s="17" t="n">
         <v>2026</v>
@@ -1753,12 +2047,12 @@
         <v>21.4</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
-        <v>59</v>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="B35" s="17" t="n">
         <v>2022</v>
@@ -1770,12 +2064,12 @@
         <v>14760.4936419221</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
-        <v>59</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="B36" s="17" t="n">
         <v>2023</v>
@@ -1787,12 +2081,12 @@
         <v>14849.0566037736</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
-        <v>59</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="B37" s="17" t="n">
         <v>2024</v>
@@ -1801,17 +2095,17 @@
         <v>14953</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="s">
-        <v>62</v>
+      <c r="A40" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B40" s="17" t="n">
         <v>2025</v>
@@ -1821,8 +2115,8 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
-        <v>62</v>
+      <c r="A41" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B41" s="17" t="n">
         <v>2026</v>
@@ -1832,8 +2126,8 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
-        <v>62</v>
+      <c r="A42" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B42" s="17" t="n">
         <v>2027</v>
@@ -1843,8 +2137,8 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="s">
-        <v>62</v>
+      <c r="A43" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B43" s="17" t="n">
         <v>2028</v>
@@ -1854,8 +2148,8 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="s">
-        <v>62</v>
+      <c r="A44" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B44" s="17" t="n">
         <v>2029</v>
@@ -1865,8 +2159,8 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="s">
-        <v>62</v>
+      <c r="A45" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B45" s="17" t="n">
         <v>2030</v>
@@ -1876,8 +2170,8 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="s">
-        <v>62</v>
+      <c r="A46" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B46" s="17" t="n">
         <v>2031</v>
@@ -1887,8 +2181,8 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
-        <v>62</v>
+      <c r="A47" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B47" s="17" t="n">
         <v>2032</v>
@@ -1898,8 +2192,8 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="s">
-        <v>62</v>
+      <c r="A48" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B48" s="17" t="n">
         <v>2033</v>
@@ -1909,8 +2203,8 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="s">
-        <v>62</v>
+      <c r="A49" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B49" s="17" t="n">
         <v>2034</v>
@@ -1920,8 +2214,8 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="s">
-        <v>62</v>
+      <c r="A50" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B50" s="17" t="n">
         <v>2035</v>
@@ -1931,8 +2225,8 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="s">
-        <v>62</v>
+      <c r="A51" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B51" s="17" t="n">
         <v>2036</v>
@@ -1942,8 +2236,8 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="s">
-        <v>62</v>
+      <c r="A52" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B52" s="17" t="n">
         <v>2037</v>
@@ -1953,8 +2247,8 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="s">
-        <v>62</v>
+      <c r="A53" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B53" s="17" t="n">
         <v>2038</v>
@@ -1964,8 +2258,8 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="s">
-        <v>62</v>
+      <c r="A54" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B54" s="17" t="n">
         <v>2039</v>
@@ -1975,8 +2269,8 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="s">
-        <v>62</v>
+      <c r="A55" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B55" s="17" t="n">
         <v>2040</v>
@@ -2025,22 +2319,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" s="24"/>
       <c r="C5" s="24"/>
@@ -2049,8 +2343,8 @@
         <v>Actualisé 2026</v>
       </c>
       <c r="E5" s="25"/>
-      <c r="G5" s="7" t="s">
-        <v>66</v>
+      <c r="G5" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="J5" s="26" t="n">
         <f aca="false">I33</f>
@@ -2059,7 +2353,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
@@ -2071,7 +2365,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="B7" s="24"/>
       <c r="C7" s="24"/>
@@ -2083,7 +2377,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B8" s="24"/>
       <c r="C8" s="24"/>
@@ -2095,7 +2389,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="24" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="B9" s="24"/>
       <c r="C9" s="24"/>
@@ -2107,7 +2401,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="B10" s="24"/>
       <c r="C10" s="24"/>
@@ -2119,7 +2413,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="B11" s="24"/>
       <c r="C11" s="24"/>
@@ -2131,7 +2425,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="24" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="B12" s="24"/>
       <c r="C12" s="24"/>
@@ -2143,46 +2437,46 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3265,28 +3559,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G3" s="3" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>90</v>
+      <c r="A4" s="5" t="s">
+        <v>108</v>
       </c>
       <c r="B4" s="37" t="n">
         <v>300000</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>91</v>
+      <c r="G4" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="H4" s="38" t="n">
         <f aca="false">B4/B6</f>
@@ -3294,14 +3588,14 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>92</v>
+      <c r="A5" s="5" t="s">
+        <v>110</v>
       </c>
       <c r="B5" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>93</v>
+      <c r="G5" s="5" t="s">
+        <v>111</v>
       </c>
       <c r="H5" s="38" t="n">
         <f aca="false">MAX(0,H4-B9)</f>
@@ -3309,14 +3603,14 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>94</v>
+      <c r="A6" s="5" t="s">
+        <v>112</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>95</v>
+      <c r="G6" s="5" t="s">
+        <v>113</v>
       </c>
       <c r="H6" s="38" t="n">
         <f aca="false">SUMPRODUCT(((H5&gt;A15:A21)*1)*(((H5&lt;B15:B21)*H5)+((H5&gt;=B15:B21)*B15:B21)-A15:A21)*C15:C21)*B6</f>
@@ -3324,14 +3618,14 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>96</v>
+      <c r="A7" s="5" t="s">
+        <v>114</v>
       </c>
       <c r="B7" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>97</v>
+      <c r="G7" s="5" t="s">
+        <v>115</v>
       </c>
       <c r="H7" s="38" t="n">
         <f aca="false">B5/B6</f>
@@ -3339,8 +3633,8 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G8" s="7" t="s">
-        <v>98</v>
+      <c r="G8" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="H8" s="38" t="n">
         <f aca="false">MAX(0,H7-B10)</f>
@@ -3348,14 +3642,14 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>99</v>
+      <c r="A9" s="5" t="s">
+        <v>117</v>
       </c>
       <c r="B9" s="39" t="n">
         <v>100000</v>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>100</v>
+      <c r="G9" s="5" t="s">
+        <v>118</v>
       </c>
       <c r="H9" s="38" t="n">
         <f aca="false">SUMPRODUCT(((H8&gt;A25:A26)*1)*(((H8&lt;B25:B26)*H8)+((H8&gt;=B25:B26)*B25:B26)-A25:A26)*C25:C26)*B6</f>
@@ -3363,14 +3657,14 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>101</v>
+      <c r="A10" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="B10" s="39" t="n">
         <v>152500</v>
       </c>
-      <c r="G10" s="7" t="s">
-        <v>102</v>
+      <c r="G10" s="5" t="s">
+        <v>120</v>
       </c>
       <c r="H10" s="40" t="n">
         <f aca="false">H6+H9</f>
@@ -3378,14 +3672,14 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>103</v>
+      <c r="A11" s="5" t="s">
+        <v>121</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>0.3</v>
       </c>
-      <c r="G11" s="7" t="s">
-        <v>104</v>
+      <c r="G11" s="5" t="s">
+        <v>122</v>
       </c>
       <c r="H11" s="38" t="n">
         <f aca="false">B4+B5</f>
@@ -3393,8 +3687,8 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G12" s="7" t="s">
-        <v>105</v>
+      <c r="G12" s="5" t="s">
+        <v>123</v>
       </c>
       <c r="H12" s="38" t="n">
         <f aca="false">SUMPRODUCT(((H11&gt;A30:A36)*1)*(((H11&lt;B30:B36)*H11)+((H11&gt;=B30:B36)*B30:B36)-A30:A36)*C30:C36)</f>
@@ -3403,10 +3697,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>107</v>
+        <v>124</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>125</v>
       </c>
       <c r="H13" s="38" t="n">
         <f aca="false">MIN(B7,B4)*B11</f>
@@ -3415,16 +3709,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>111</v>
+        <v>128</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>129</v>
       </c>
       <c r="H14" s="40" t="n">
         <f aca="false">H12+H13</f>
@@ -3441,8 +3735,8 @@
       <c r="C15" s="14" t="n">
         <v>0.05</v>
       </c>
-      <c r="G15" s="7" t="s">
-        <v>112</v>
+      <c r="G15" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="H15" s="40" t="n">
         <f aca="false">H14-H10</f>
@@ -3459,8 +3753,8 @@
       <c r="C16" s="14" t="n">
         <v>0.1</v>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>113</v>
+      <c r="G16" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="H16" s="33" t="n">
         <f aca="false">IF(H11&gt;0,H10/H11,0)</f>
@@ -3477,8 +3771,8 @@
       <c r="C17" s="14" t="n">
         <v>0.15</v>
       </c>
-      <c r="G17" s="7" t="s">
-        <v>114</v>
+      <c r="G17" s="5" t="s">
+        <v>132</v>
       </c>
       <c r="H17" s="33" t="n">
         <f aca="false">IF(H11&gt;0,H14/H11,0)</f>
@@ -3507,7 +3801,7 @@
         <v>0.3</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3534,18 +3828,18 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3572,18 +3866,18 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3689,74 +3983,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>121</v>
+      <c r="A4" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>122</v>
+      <c r="A5" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>123</v>
+      <c r="A6" s="5" t="s">
+        <v>141</v>
       </c>
       <c r="B6" s="37" t="n">
         <v>2100</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>124</v>
+      <c r="A8" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="B8" s="41" t="n">
         <v>30400000</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>126</v>
+      <c r="A9" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="B9" s="42" t="n">
         <v>1108500000000</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>128</v>
+      <c r="A10" s="5" t="s">
+        <v>146</v>
       </c>
       <c r="B10" s="11" t="n">
         <v>0.78</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>130</v>
+      <c r="A12" s="5" t="s">
+        <v>148</v>
       </c>
       <c r="B12" s="43" t="n">
         <f aca="false">IF(B4="Moyenne",'Modèle IGS'!D10,INDEX('Modèle IGS'!M18:M33,MATCH(VALUE(B4),'Modèle IGS'!A18:A33,0)))</f>
@@ -3764,8 +4058,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>131</v>
+      <c r="A13" s="5" t="s">
+        <v>149</v>
       </c>
       <c r="B13" s="44" t="n">
         <f aca="false">B12*B5</f>
@@ -3773,8 +4067,8 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>132</v>
+      <c r="A14" s="5" t="s">
+        <v>150</v>
       </c>
       <c r="B14" s="45" t="n">
         <f aca="false">B13*1000000000/B8/12</f>
@@ -3782,8 +4076,8 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>133</v>
+      <c r="A15" s="5" t="s">
+        <v>151</v>
       </c>
       <c r="B15" s="45" t="n">
         <f aca="false">B13*1000000000*(B6*12/B10)/B9/12</f>
@@ -3822,121 +4116,121 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="C4" s="46" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="C6" s="46" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="C7" s="46" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="C8" s="46" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="C14" s="46" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -3955,4 +4249,329 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="F5" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F6" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F7" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F8" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F9" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F10" s="47" t="s">
+        <v>159</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="F11" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F12" s="47" t="s">
+        <v>165</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="F13" s="47" t="s">
+        <v>215</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="F14" s="47" t="s">
+        <v>220</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F5" r:id="rId1" display="https://www.legifrance.gouv.fr/codes/texte_lc/LEGITEXT000006069577"/>
+    <hyperlink ref="F6" r:id="rId2" display="https://www.legifrance.gouv.fr/codes/texte_lc/LEGITEXT000006069577"/>
+    <hyperlink ref="F7" r:id="rId3" display="https://www.jean-jaures.org/publication/face-a-la-grande-transmission-limpot-sur-les-grandes-successions/"/>
+    <hyperlink ref="F8" r:id="rId4" display="https://www.jean-jaures.org/publication/face-a-la-grande-transmission-limpot-sur-les-grandes-successions/"/>
+    <hyperlink ref="F9" r:id="rId5" display="https://www.jean-jaures.org/publication/face-a-la-grande-transmission-limpot-sur-les-grandes-successions/"/>
+    <hyperlink ref="F10" r:id="rId6" display="https://www.insee.fr/fr/statistiques/8996855"/>
+    <hyperlink ref="F11" r:id="rId7" display="https://www.assemblee-nationale.fr/dyn/contenu/visualisation/1087930/file/PLF%202026%20-%20V%26M%20TI%20-%20Evaluations%20des%20recettes.pdf"/>
+    <hyperlink ref="F12" r:id="rId8" display="https://www.insee.fr/fr/statistiques/8661938"/>
+    <hyperlink ref="F13" r:id="rId9" display="https://placement.meilleurtaux.com/placement-financier/actualites/2026-avril/flat-tax-a-31-4-ce-qui-change-depuis-janvier-2026.html"/>
+    <hyperlink ref="F14" r:id="rId10" display="https://www.insee.fr/fr/statistiques/8376894"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Vérification des chiffres des classeurs ; TVA : perte de pouvoir d'achat lue sur le graphique 4 du Trésor-Éco (#18)
- TVA sociale : la perte par point de taux normal n'est plus le prorata 0,5 % × 8,9 / 13,7 (0,325 %) mais les
  valeurs du graphique 4 du Trésor-Éco n° 371, par cinquième de niveau de vie (0,39 % à 0,25 % ; moyenne 0,30 %),
  avec le choix du cinquième dans le simulateur et le classeur.
- Classeurs : feuille « Vérification » (type, calcul, source, lien, statut de chaque chiffre saisi), colonnes « Type »
  et « Comment c'est calculé » dans les tableaux de paramètres, source Insee dans la feuille Niveaux de vie.
- Registre tools/chiffrages/verification.py.


Claude-Session: https://claude.ai/code/session_0188qNw1StBQkFA1rFcQwdyx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/chiffrages/Chiffrage_Heritage.xlsx
+++ b/site/chiffrages/Chiffrage_Heritage.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Calcul individuel" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Gain salaire" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Sources" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Vérification" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="223">
   <si>
     <t xml:space="preserve">Chiffrage de l'espace Héritage</t>
   </si>
@@ -85,6 +86,9 @@
     <t xml:space="preserve">L'étude mêle euros courants et croissances réelles (PIB +1 %/an sans inflation) ; la part du top 1 % du patrimoine y passe de 24 % à 35 % en 2040 ; aucun effet de comportement (exil, optimisation, étalement du paiement).</t>
   </si>
   <si>
+    <t xml:space="preserve">Chaque chiffre saisi est revérifié à la source : voir la feuille « Vérification » (type, calcul, source, statut).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Légende des couleurs</t>
   </si>
   <si>
@@ -133,39 +137,75 @@
     <t xml:space="preserve">Source</t>
   </si>
   <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment c'est calculé</t>
+  </si>
+  <si>
     <t xml:space="preserve">Croissance annuelle du PIB (après la dernière année connue)</t>
   </si>
   <si>
     <t xml:space="preserve">Étude : +1 % par an</t>
   </si>
   <si>
+    <t xml:space="preserve">Hypothèse du site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypothèse de l'étude : +1 % par an après la dernière année connue.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Flux successoral en 2050 (part du PIB)</t>
   </si>
   <si>
     <t xml:space="preserve">CAE, note n° 63, 2021 (d'après Goupille-Lebret et al.)</t>
   </si>
   <si>
+    <t xml:space="preserve">Chiffre publié</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 % du PIB en 2050 (CAE, note n° 63) ; interpolation linéaire depuis 15 % en 2021.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Croissance annuelle du patrimoine du top 1 %</t>
   </si>
   <si>
     <t xml:space="preserve">Garbinti, Goupille-Lebret et Piketty (2021) : 6,10 % par an en moyenne sur 2005-2014, moins 2 % d'inflation</t>
   </si>
   <si>
+    <t xml:space="preserve">Calcul du site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,10 % de rendement moyen 2005-2014 (Garbinti et al.) − 2 % d'inflation.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part de plus-values latentes dans le patrimoine du top 1 %</t>
   </si>
   <si>
     <t xml:space="preserve">Saez et al. (2021) : 17 681 Md€ de plus-values latentes sur 42 861 Md€ de patrimoine du top 1 %</t>
   </si>
   <si>
+    <t xml:space="preserve">17 681 Md€ de plus-values latentes ÷ 42 861 Md€ de patrimoine du top 1 % (Saez et al.).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Taux du PFU</t>
   </si>
   <si>
     <t xml:space="preserve">PFU de 30 % (2024) / PFU de 31,4 % depuis le 1er janvier 2026 (12,8 % d'impôt + 18,6 % de prélèvements sociaux, LFSS 2026)</t>
   </si>
   <si>
+    <t xml:space="preserve">Loi ou barème</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 % en 2024 ; 31,4 % depuis 2026 (12,8 % + 18,6 %).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Flux successoral en 2021 (part du PIB)</t>
   </si>
   <si>
+    <t xml:space="preserve">15 % du PIB en 2021 (CAE, note n° 63).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Année de départ du flux</t>
   </si>
   <si>
@@ -178,12 +218,18 @@
     <t xml:space="preserve">CAE (2021), simulation de la réforme de l'assiette et du barème, reprise par l'étude</t>
   </si>
   <si>
+    <t xml:space="preserve">10 Md€ en 2021 (simulation du CAE reprise par l'étude), puis comme le flux successoral.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part du patrimoine détenue par le top 1 % (année de référence)</t>
   </si>
   <si>
     <t xml:space="preserve">World Inequality Database, 2022</t>
   </si>
   <si>
+    <t xml:space="preserve">24 % (World Inequality Database, 2022).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Année de référence du patrimoine du top 1 %</t>
   </si>
   <si>
@@ -193,18 +239,27 @@
     <t xml:space="preserve">4,07 % − 2 % d'inflation (étude, Banque de France)</t>
   </si>
   <si>
+    <t xml:space="preserve">4,07 % − 2 % d'inflation (classeur de l'étude, Banque de France).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part de l'assiette taxée après abattements</t>
   </si>
   <si>
     <t xml:space="preserve">Hannezo et al. (2022)</t>
   </si>
   <si>
+    <t xml:space="preserve">80 % de l'assiette taxée (Hannezo et al., 2022).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réduction pour droits de succession déjà payés</t>
   </si>
   <si>
     <t xml:space="preserve">CAE (2021)</t>
   </si>
   <si>
+    <t xml:space="preserve">20 % de droits déjà payés déduits (CAE, 2021).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Données connues par année (au-delà : projection)</t>
   </si>
   <si>
@@ -518,6 +573,150 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.insee.fr/fr/statistiques/8574681?sommaire=8574832</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérification des chiffres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chaque chiffre saisi dans ce classeur, revérifié à la source en octobre 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remarque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème en ligne directe (5 % à 45 %, tranches de 8 072 à 1 805 677 €) et abattement de 100 000 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème légal, inchangé depuis 2011.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGI, art. 777 et 779</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.legifrance.gouv.fr/codes/texte_lc/LEGITEXT000006069577</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'étude écrit « 15 392 € » pour la borne de la tranche à 15 % ; le bon chiffre, retenu ici, est 15 932 €.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assurance-vie : abattement de 152 500 € par bénéficiaire, 20 % jusqu'à 700 000 €, 31,25 % au-delà</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primes versées avant 70 ans.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGI, art. 990 I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème de l'IGS (0 % jusqu'à 200 000 €, puis 5 / 15 / 25 / 35 / 45 / 50 %)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau 6 de l'étude (proposition du CAE, 2021).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fondation Jean-Jaurès (2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PFU sur les plus-values latentes (calcul individuel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux de l'étude (2024) ; 31,4 % depuis 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flux successoral, pilier 1, pilier 2 : formules et hypothèses du scénario « Étude 2024 »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repris du classeur de chiffrage de l'étude, cellule par cellule (vérifié : mêmes résultats à 0,01 Md€ près).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fondation Jean-Jaurès (2024), classeur « Chiffrage IGS »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIB 2025 (scénario actualisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 991,1 Md€</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024 déduit : 2 991,1 ÷ 1,019 (croissance en valeur de 1,9 %).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insee, Les comptes de la Nation en 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Droits de succession et donations 2024-2026 (scénario actualisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20,9 ; 20,7 ; 21,4 Md€</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donations + successions : 4,9 + 16,0 ; 4,5 + 16,2 ; 4,4 + 17,0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voies et moyens, PLF 2026, tome I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrimoine net des ménages (scénario actualisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 953 Md€ fin 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023 et 2022 déduits des évolutions publiées (+0,7 %, +0,6 %).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insee Première n° 2081</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PFU (scénario actualisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31,4 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12,8 % d'impôt + 18,6 % de prélèvements sociaux depuis le 1er janvier 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LFSS 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://placement.meilleurtaux.com/placement-financier/actualites/2026-avril/flat-tax-a-31-4-ce-qui-change-depuis-janvier-2026.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnes en emploi ; salaires bruts ; ratio net / brut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30,4 M ; 1 108,5 Md€ ; 78 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voir le classeur Retraites (ratio : hypothèse du site).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.insee.fr/fr/statistiques/8376894</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Types : « Chiffre publié » (repris d'une publication), « Lu sur un graphique », « Calcul du site » (formule à partir de chiffres publiés), « Hypothèse du site », « Loi ou barème ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statuts : « Confirmé » (vérifié à la source primaire), « Corrigé » (valeur changée lors de cette vérification), « Confirmé (source secondaire) », « Estimation, non vérifiable ».</t>
   </si>
 </sst>
 </file>
@@ -695,7 +894,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -716,6 +915,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -724,10 +927,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -882,6 +1081,10 @@
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1136,7 +1339,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1203,33 +1406,38 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1248,62 +1456,70 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="B4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="n">
         <f aca="false">IF(B4="Étude 2024",1,2)</f>
         <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>0.01</v>
@@ -1317,12 +1533,18 @@
         <v>0.01</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>32</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>0.23</v>
@@ -1336,12 +1558,18 @@
         <v>0.23</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>0.041</v>
@@ -1355,12 +1583,18 @@
         <v>0.041</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>40</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>0.412519539908075</v>
@@ -1374,12 +1608,18 @@
         <v>0.412519539908075</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>35</v>
+        <v>44</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>0.3</v>
@@ -1393,12 +1633,18 @@
         <v>0.314</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>37</v>
+        <v>47</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="B12" s="11" t="n">
         <v>0.15</v>
@@ -1412,12 +1658,18 @@
         <v>0.15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>31</v>
+        <v>36</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>2021</v>
@@ -1431,10 +1683,14 @@
         <v>2021</v>
       </c>
       <c r="F13" s="4"/>
+      <c r="G13" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>2050</v>
@@ -1448,10 +1704,14 @@
         <v>2050</v>
       </c>
       <c r="F14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G14" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B15" s="20" t="n">
         <v>10</v>
@@ -1465,12 +1725,18 @@
         <v>10</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>42</v>
+        <v>55</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>0.24</v>
@@ -1484,12 +1750,18 @@
         <v>0.24</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>44</v>
+        <v>58</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>2022</v>
@@ -1503,10 +1775,14 @@
         <v>2022</v>
       </c>
       <c r="F17" s="4"/>
+      <c r="G17" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>0.0207</v>
@@ -1520,12 +1796,18 @@
         <v>0.0207</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>47</v>
+        <v>62</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="B19" s="11" t="n">
         <v>0.8</v>
@@ -1539,12 +1821,18 @@
         <v>0.8</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>49</v>
+        <v>65</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="B20" s="11" t="n">
         <v>0.2</v>
@@ -1558,35 +1846,41 @@
         <v>0.2</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>51</v>
+        <v>68</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>55</v>
+      <c r="A24" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>2021</v>
@@ -1598,12 +1892,12 @@
         <v>2508.1023</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>55</v>
+      <c r="A25" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B25" s="17" t="n">
         <v>2022</v>
@@ -1615,12 +1909,12 @@
         <v>2655.435</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>55</v>
+      <c r="A26" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B26" s="17" t="n">
         <v>2023</v>
@@ -1632,12 +1926,12 @@
         <v>2822.5</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
-        <v>55</v>
+      <c r="A27" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B27" s="17" t="n">
         <v>2024</v>
@@ -1646,12 +1940,12 @@
         <v>2935.32875368008</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>55</v>
+      <c r="A28" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B28" s="17" t="n">
         <v>2025</v>
@@ -1660,12 +1954,12 @@
         <v>2991.1</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
-        <v>57</v>
+      <c r="A29" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B29" s="17" t="n">
         <v>2021</v>
@@ -1677,12 +1971,12 @@
         <v>18.7</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
-        <v>57</v>
+      <c r="A30" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B30" s="17" t="n">
         <v>2022</v>
@@ -1694,12 +1988,12 @@
         <v>18.7</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
-        <v>57</v>
+      <c r="A31" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B31" s="17" t="n">
         <v>2023</v>
@@ -1711,12 +2005,12 @@
         <v>20.8</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>57</v>
+      <c r="A32" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B32" s="17" t="n">
         <v>2024</v>
@@ -1725,12 +2019,12 @@
         <v>20.9</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>57</v>
+      <c r="A33" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B33" s="17" t="n">
         <v>2025</v>
@@ -1739,12 +2033,12 @@
         <v>20.7</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
-        <v>57</v>
+      <c r="A34" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B34" s="17" t="n">
         <v>2026</v>
@@ -1753,12 +2047,12 @@
         <v>21.4</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
-        <v>59</v>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="B35" s="17" t="n">
         <v>2022</v>
@@ -1770,12 +2064,12 @@
         <v>14760.4936419221</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
-        <v>59</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="B36" s="17" t="n">
         <v>2023</v>
@@ -1787,12 +2081,12 @@
         <v>14849.0566037736</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
-        <v>59</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="B37" s="17" t="n">
         <v>2024</v>
@@ -1801,17 +2095,17 @@
         <v>14953</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="s">
-        <v>62</v>
+      <c r="A40" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B40" s="17" t="n">
         <v>2025</v>
@@ -1821,8 +2115,8 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
-        <v>62</v>
+      <c r="A41" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B41" s="17" t="n">
         <v>2026</v>
@@ -1832,8 +2126,8 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
-        <v>62</v>
+      <c r="A42" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B42" s="17" t="n">
         <v>2027</v>
@@ -1843,8 +2137,8 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="s">
-        <v>62</v>
+      <c r="A43" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B43" s="17" t="n">
         <v>2028</v>
@@ -1854,8 +2148,8 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="s">
-        <v>62</v>
+      <c r="A44" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B44" s="17" t="n">
         <v>2029</v>
@@ -1865,8 +2159,8 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="s">
-        <v>62</v>
+      <c r="A45" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B45" s="17" t="n">
         <v>2030</v>
@@ -1876,8 +2170,8 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="s">
-        <v>62</v>
+      <c r="A46" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B46" s="17" t="n">
         <v>2031</v>
@@ -1887,8 +2181,8 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
-        <v>62</v>
+      <c r="A47" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B47" s="17" t="n">
         <v>2032</v>
@@ -1898,8 +2192,8 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="s">
-        <v>62</v>
+      <c r="A48" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B48" s="17" t="n">
         <v>2033</v>
@@ -1909,8 +2203,8 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="s">
-        <v>62</v>
+      <c r="A49" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B49" s="17" t="n">
         <v>2034</v>
@@ -1920,8 +2214,8 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="s">
-        <v>62</v>
+      <c r="A50" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B50" s="17" t="n">
         <v>2035</v>
@@ -1931,8 +2225,8 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="s">
-        <v>62</v>
+      <c r="A51" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B51" s="17" t="n">
         <v>2036</v>
@@ -1942,8 +2236,8 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="s">
-        <v>62</v>
+      <c r="A52" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B52" s="17" t="n">
         <v>2037</v>
@@ -1953,8 +2247,8 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="s">
-        <v>62</v>
+      <c r="A53" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B53" s="17" t="n">
         <v>2038</v>
@@ -1964,8 +2258,8 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="s">
-        <v>62</v>
+      <c r="A54" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B54" s="17" t="n">
         <v>2039</v>
@@ -1975,8 +2269,8 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="s">
-        <v>62</v>
+      <c r="A55" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B55" s="17" t="n">
         <v>2040</v>
@@ -2025,22 +2319,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" s="24"/>
       <c r="C5" s="24"/>
@@ -2049,8 +2343,8 @@
         <v>Actualisé 2026</v>
       </c>
       <c r="E5" s="25"/>
-      <c r="G5" s="7" t="s">
-        <v>66</v>
+      <c r="G5" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="J5" s="26" t="n">
         <f aca="false">I33</f>
@@ -2059,7 +2353,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
@@ -2071,7 +2365,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="B7" s="24"/>
       <c r="C7" s="24"/>
@@ -2083,7 +2377,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B8" s="24"/>
       <c r="C8" s="24"/>
@@ -2095,7 +2389,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="24" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="B9" s="24"/>
       <c r="C9" s="24"/>
@@ -2107,7 +2401,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="B10" s="24"/>
       <c r="C10" s="24"/>
@@ -2119,7 +2413,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="B11" s="24"/>
       <c r="C11" s="24"/>
@@ -2131,7 +2425,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="24" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="B12" s="24"/>
       <c r="C12" s="24"/>
@@ -2143,46 +2437,46 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3265,28 +3559,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G3" s="3" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>90</v>
+      <c r="A4" s="5" t="s">
+        <v>108</v>
       </c>
       <c r="B4" s="37" t="n">
         <v>300000</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>91</v>
+      <c r="G4" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="H4" s="38" t="n">
         <f aca="false">B4/B6</f>
@@ -3294,14 +3588,14 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>92</v>
+      <c r="A5" s="5" t="s">
+        <v>110</v>
       </c>
       <c r="B5" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>93</v>
+      <c r="G5" s="5" t="s">
+        <v>111</v>
       </c>
       <c r="H5" s="38" t="n">
         <f aca="false">MAX(0,H4-B9)</f>
@@ -3309,14 +3603,14 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>94</v>
+      <c r="A6" s="5" t="s">
+        <v>112</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>95</v>
+      <c r="G6" s="5" t="s">
+        <v>113</v>
       </c>
       <c r="H6" s="38" t="n">
         <f aca="false">SUMPRODUCT(((H5&gt;A15:A21)*1)*(((H5&lt;B15:B21)*H5)+((H5&gt;=B15:B21)*B15:B21)-A15:A21)*C15:C21)*B6</f>
@@ -3324,14 +3618,14 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>96</v>
+      <c r="A7" s="5" t="s">
+        <v>114</v>
       </c>
       <c r="B7" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>97</v>
+      <c r="G7" s="5" t="s">
+        <v>115</v>
       </c>
       <c r="H7" s="38" t="n">
         <f aca="false">B5/B6</f>
@@ -3339,8 +3633,8 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G8" s="7" t="s">
-        <v>98</v>
+      <c r="G8" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="H8" s="38" t="n">
         <f aca="false">MAX(0,H7-B10)</f>
@@ -3348,14 +3642,14 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>99</v>
+      <c r="A9" s="5" t="s">
+        <v>117</v>
       </c>
       <c r="B9" s="39" t="n">
         <v>100000</v>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>100</v>
+      <c r="G9" s="5" t="s">
+        <v>118</v>
       </c>
       <c r="H9" s="38" t="n">
         <f aca="false">SUMPRODUCT(((H8&gt;A25:A26)*1)*(((H8&lt;B25:B26)*H8)+((H8&gt;=B25:B26)*B25:B26)-A25:A26)*C25:C26)*B6</f>
@@ -3363,14 +3657,14 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>101</v>
+      <c r="A10" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="B10" s="39" t="n">
         <v>152500</v>
       </c>
-      <c r="G10" s="7" t="s">
-        <v>102</v>
+      <c r="G10" s="5" t="s">
+        <v>120</v>
       </c>
       <c r="H10" s="40" t="n">
         <f aca="false">H6+H9</f>
@@ -3378,14 +3672,14 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>103</v>
+      <c r="A11" s="5" t="s">
+        <v>121</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>0.3</v>
       </c>
-      <c r="G11" s="7" t="s">
-        <v>104</v>
+      <c r="G11" s="5" t="s">
+        <v>122</v>
       </c>
       <c r="H11" s="38" t="n">
         <f aca="false">B4+B5</f>
@@ -3393,8 +3687,8 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G12" s="7" t="s">
-        <v>105</v>
+      <c r="G12" s="5" t="s">
+        <v>123</v>
       </c>
       <c r="H12" s="38" t="n">
         <f aca="false">SUMPRODUCT(((H11&gt;A30:A36)*1)*(((H11&lt;B30:B36)*H11)+((H11&gt;=B30:B36)*B30:B36)-A30:A36)*C30:C36)</f>
@@ -3403,10 +3697,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>107</v>
+        <v>124</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>125</v>
       </c>
       <c r="H13" s="38" t="n">
         <f aca="false">MIN(B7,B4)*B11</f>
@@ -3415,16 +3709,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>111</v>
+        <v>128</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>129</v>
       </c>
       <c r="H14" s="40" t="n">
         <f aca="false">H12+H13</f>
@@ -3441,8 +3735,8 @@
       <c r="C15" s="14" t="n">
         <v>0.05</v>
       </c>
-      <c r="G15" s="7" t="s">
-        <v>112</v>
+      <c r="G15" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="H15" s="40" t="n">
         <f aca="false">H14-H10</f>
@@ -3459,8 +3753,8 @@
       <c r="C16" s="14" t="n">
         <v>0.1</v>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>113</v>
+      <c r="G16" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="H16" s="33" t="n">
         <f aca="false">IF(H11&gt;0,H10/H11,0)</f>
@@ -3477,8 +3771,8 @@
       <c r="C17" s="14" t="n">
         <v>0.15</v>
       </c>
-      <c r="G17" s="7" t="s">
-        <v>114</v>
+      <c r="G17" s="5" t="s">
+        <v>132</v>
       </c>
       <c r="H17" s="33" t="n">
         <f aca="false">IF(H11&gt;0,H14/H11,0)</f>
@@ -3507,7 +3801,7 @@
         <v>0.3</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3534,18 +3828,18 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3572,18 +3866,18 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3689,74 +3983,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>121</v>
+      <c r="A4" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>122</v>
+      <c r="A5" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>123</v>
+      <c r="A6" s="5" t="s">
+        <v>141</v>
       </c>
       <c r="B6" s="37" t="n">
         <v>2100</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>124</v>
+      <c r="A8" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="B8" s="41" t="n">
         <v>30400000</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>126</v>
+      <c r="A9" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="B9" s="42" t="n">
         <v>1108500000000</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>128</v>
+      <c r="A10" s="5" t="s">
+        <v>146</v>
       </c>
       <c r="B10" s="11" t="n">
         <v>0.78</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>130</v>
+      <c r="A12" s="5" t="s">
+        <v>148</v>
       </c>
       <c r="B12" s="43" t="n">
         <f aca="false">IF(B4="Moyenne",'Modèle IGS'!D10,INDEX('Modèle IGS'!M18:M33,MATCH(VALUE(B4),'Modèle IGS'!A18:A33,0)))</f>
@@ -3764,8 +4058,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>131</v>
+      <c r="A13" s="5" t="s">
+        <v>149</v>
       </c>
       <c r="B13" s="44" t="n">
         <f aca="false">B12*B5</f>
@@ -3773,8 +4067,8 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>132</v>
+      <c r="A14" s="5" t="s">
+        <v>150</v>
       </c>
       <c r="B14" s="45" t="n">
         <f aca="false">B13*1000000000/B8/12</f>
@@ -3782,8 +4076,8 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>133</v>
+      <c r="A15" s="5" t="s">
+        <v>151</v>
       </c>
       <c r="B15" s="45" t="n">
         <f aca="false">B13*1000000000*(B6*12/B10)/B9/12</f>
@@ -3822,121 +4116,121 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="C4" s="46" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="C6" s="46" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="C7" s="46" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="C8" s="46" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="C14" s="46" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -3955,4 +4249,329 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="F5" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F6" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F7" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F8" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F9" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F10" s="47" t="s">
+        <v>159</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="F11" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F12" s="47" t="s">
+        <v>165</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="F13" s="47" t="s">
+        <v>215</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="F14" s="47" t="s">
+        <v>220</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F5" r:id="rId1" display="https://www.legifrance.gouv.fr/codes/texte_lc/LEGITEXT000006069577"/>
+    <hyperlink ref="F6" r:id="rId2" display="https://www.legifrance.gouv.fr/codes/texte_lc/LEGITEXT000006069577"/>
+    <hyperlink ref="F7" r:id="rId3" display="https://www.jean-jaures.org/publication/face-a-la-grande-transmission-limpot-sur-les-grandes-successions/"/>
+    <hyperlink ref="F8" r:id="rId4" display="https://www.jean-jaures.org/publication/face-a-la-grande-transmission-limpot-sur-les-grandes-successions/"/>
+    <hyperlink ref="F9" r:id="rId5" display="https://www.jean-jaures.org/publication/face-a-la-grande-transmission-limpot-sur-les-grandes-successions/"/>
+    <hyperlink ref="F10" r:id="rId6" display="https://www.insee.fr/fr/statistiques/8996855"/>
+    <hyperlink ref="F11" r:id="rId7" display="https://www.assemblee-nationale.fr/dyn/contenu/visualisation/1087930/file/PLF%202026%20-%20V%26M%20TI%20-%20Evaluations%20des%20recettes.pdf"/>
+    <hyperlink ref="F12" r:id="rId8" display="https://www.insee.fr/fr/statistiques/8661938"/>
+    <hyperlink ref="F13" r:id="rId9" display="https://placement.meilleurtaux.com/placement-financier/actualites/2026-avril/flat-tax-a-31-4-ce-qui-change-depuis-janvier-2026.html"/>
+    <hyperlink ref="F14" r:id="rId10" display="https://www.insee.fr/fr/statistiques/8376894"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>